<commit_message>
fix: honest audit of B6 Laporan Akses 2026 and route aliases
</commit_message>
<xml_diff>
--- a/SPREADSHEET_PENILAIAN_AKIP_2026_REVISI_TERBARU_PKTJ.xlsx
+++ b/SPREADSHEET_PENILAIAN_AKIP_2026_REVISI_TERBARU_PKTJ.xlsx
@@ -1043,29 +1043,30 @@
           <t>Jumlah permohonan informasi yang diminta</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>Ya (Lengkap)</t>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Parsial (Perlu Unggah Berkas)</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Portal /layanan/laporan-akses menampilkan visualisasi statistik dan rekapitulasi jumlah permohonan bulanan 2024-2026.</t>
+          <t>Struktur menu /layanan-informasi/laporan sudah aktif di web, namun dokumen tabel laporan bulanan/tahunan TA 2026 belum diunggah.</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>https://ppid.pktj.ac.id/layanan-informasi/laporan (catatan: laporan bulanan agustus dibuat dicapture dibuatkan notadinas)</t>
+          <t>laporan bulanan agustus dibuat dicapture dibuatkan notadinas ke PPID pelaksana ditembuskan ke PPID Utama (Link: https://ppid.pktj.ac.id/layanan-informasi/laporan)</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>SESUAI &amp; VALID: Data permohonan telah tayang interaktif.</t>
+          <t>SEGERA DILENGKAPI: File rekapitulasi/capture laporan bulanan permohonan informasi TA 2026 beserta Nota Dinas wajib di-upload ke menu Layanan Informasi atau folder Drive AKIP.</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>https://ppid.pktj.ac.id/layanan/laporan-akses</t>
+          <t>https://ppid.pktj.ac.id/layanan-informasi/laporan
+(Folder Drive Laporan: https://drive.google.com/drive/folders/12XsoBWqjqXErm1puxuZmtQMDo-UBad5n)</t>
         </is>
       </c>
     </row>
@@ -1087,27 +1088,28 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Ya (Lengkap)</t>
+          <t>Ya (SOP Ada, Rekap Bulanan di Laporan)</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Laporan Akses menyajikan rata-rata waktu pemenuhan (standar &lt; 10 hari kerja + perpanjangan 7 hari kerja).</t>
+          <t>Standar waktu pelayanan tertuang di SOP Standar Waktu (&lt; 10 hari kerja + perpanjangan 7 hari kerja). Realisasi waktu pemenuhan bulanan wajib dimuat dalam laporan bulanan.</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>https://ppid.pktj.ac.id/layanan-informasi/laporan (catatan: form permohonan ditambah KTP)</t>
+          <t>pada form permohonan lewat google form ditambah KTP (Link: https://ppid.pktj.ac.id/layanan-informasi/laporan)</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>SESUAI &amp; VALID: Formulir online sudah mewajibkan unggah identitas KTP/SIM.</t>
+          <t>SESUAI: SOP standar waktu tayang di web. Data riil waktu pemenuhan bulanan dituangkan dalam laporan bulanan permohonan informasi.</t>
         </is>
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t>https://ppid.pktj.ac.id/layanan/laporan-akses</t>
+          <t>https://ppid.pktj.ac.id/prosedur/sop-standar-waktu
+(Laporan: https://ppid.pktj.ac.id/layanan-informasi/laporan)</t>
         </is>
       </c>
     </row>
@@ -1127,29 +1129,29 @@
           <t>Jumlah permohonan informasi publik yang dikabulkan baik sebagian atau seluruhnya dan yang ditolak</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>Ya (Lengkap)</t>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Parsial (Perlu Rekap Bulanan)</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Rekapitulasi status pemenuhan (dikabulkan / ditolak) ditampilkan transparan di halaman Laporan Akses.</t>
+          <t>Data rekapitulasi status permohonan (dikabulkan / ditolak) TA 2026 perlu dituangkan dalam rekap laporan bulanan PPID.</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>https://ppid.pktj.ac.id/layanan-informasi/laporan (catatan: Maklumat dicetak di ruang PPID)</t>
+          <t>Maklumat PPID dibuat, dicetak, taruh di ruang PPID (Link: https://ppid.pktj.ac.id/layanan-informasi/laporan)</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>SESUAI &amp; VALID: Rincian status tampil di website.</t>
+          <t>SEGERA DILENGKAPI: Rekapitulasi permohonan dikabulkan/ditolak disatukan dalam berkas laporan bulanan permohonan informasi TA 2026.</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>https://ppid.pktj.ac.id/layanan/laporan-akses</t>
+          <t>https://ppid.pktj.ac.id/layanan-informasi/laporan</t>
         </is>
       </c>
     </row>
@@ -1171,28 +1173,28 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Ya (Lengkap)</t>
+          <t>Ya (Dasar Hukum Terbit, Kasus di Laporan)</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Alasan penolakan tercantum di Laporan Akses dan mengacu pada 7 Dokumen Informasi Dikecualikan (DIK) yang telah diuji konsekuensi (ID: 726).</t>
+          <t>Landasan penolakan mengacu pada 7 Dokumen Informasi Dikecualikan (DIK) hasil uji konsekuensi (ID: 726). Rekapitulasi kasus penolakan dituangkan di laporan bulanan.</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>https://ppid.pktj.ac.id/layanan-informasi/laporan (catatan: untuk LSM wajib KTP dan Akta pendirian LSM)</t>
+          <t>untuk LSM wajib KTP dan Akta pendirian LSM (Link: https://ppid.pktj.ac.id/layanan-informasi/laporan)</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>SESUAI &amp; VALID: Persyaratan LSM sudah dicantumkan dalam syarat permohonan.</t>
+          <t>SESUAI: Regulasi &amp; DIP Dikecualikan tayang di web. Persyaratan penolakan (misal pemohon tanpa KTP/Akta LSM) tertuang di SOP &amp; form.</t>
         </is>
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>https://ppid.pktj.ac.id/layanan/laporan-akses
-(DIP Dikecualikan: https://ppid.pktj.ac.id/informasi-publik/dikecualikan)</t>
+          <t>https://ppid.pktj.ac.id/informasi-publik/dikecualikan
+(Laporan: https://ppid.pktj.ac.id/layanan-informasi/laporan)</t>
         </is>
       </c>
     </row>
@@ -1214,22 +1216,22 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Ya (Lengkap)</t>
+          <t>Ya (Lengkap di Google Drive)</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Laporan Layanan Informasi Publik 2025 dan bukti tanda terima/pengantar ke PPID Utama tersimpan di Google Drive.</t>
+          <t>Laporan Layanan Informasi Publik 2025 dan bukti tanda terima/surat pengantar ke PPID Utama Dephub tersimpan di Google Drive.</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/12XsoBWqjqXErm1puxuZmtQMDo-UBad5n?usp=drive_link (catatan: Surat DIP dan DIK 2025 kemenhub dimasukkan)</t>
+          <t>Surat DIP dan DIK 2025 kemenhub tolong dimasukkan (Link Drive: 12XsoBWqjqXErm1puxuZmtQMDo-UBad5n)</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>SESUAI &amp; VALID: File laporan dan bukti kirim ke PPID Utama tersedia di Drive.</t>
+          <t>SESUAI &amp; VALID: File laporan dan bukti kirim ke PPID Utama sudah ada di Google Drive data dukung.</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
@@ -1254,14 +1256,14 @@
           <t>Apakah unit kerja saudara mengumumkan laporan akses informasi publik tahun 2026 (Laporan bulanan permohonan informasi) di website?</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
-        <is>
-          <t>Ya (Lengkap)</t>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>BELUM ADA (BELUM DIUNGGAH KE WEBSITE)</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Halaman /layanan/laporan-akses SUDAH AKTIF dan menyajikan data bulanan berjalan 2026 secara transparan.</t>
+          <t>Dokumen file/PDF Laporan Akses Informasi Publik TA 2026 (laporan bulanan permohonan informasi 2026) BELUM ADA SAMA SEKALI di website (di database, jumlah berkas dokumen laporan akses saat ini masih 0).</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1271,12 +1273,12 @@
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>KOREKSI ATAS CATATAN REKAN: Rekan mencatat 'BELUM DIMASUKKAN', padahal halaman /layanan/laporan-akses SUDAH TERSEDIA dan aktif menampilkan rekap 2026!</t>
+          <t>CATATAN REKAN 100% BENAR &amp; VALID: Laporan bulanan permohonan informasi TA 2026 (seperti capture rekap bulanan Januari–Agustus 2026 beserta Nota Dinas ke PPID Pelaksana/Utama) MEMANG BELUM DIMASUKKAN KE WEBSITE. TINDAK LANJUT WAJIB: Petugas Meja Layanan PPID segera menyusun file PDF rekap laporan bulanan permohonan informasi TA 2026, lalu Admin PPID wajib mengunggah file tersebut ke menu Layanan Informasi dan melampirkan link Drive resminya sebelum batas submit AKIP 30 September 2026.</t>
         </is>
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>https://ppid.pktj.ac.id/layanan/laporan-akses</t>
+          <t>BELUM ADA DI WEBSITE (Wajib Segera Disusun &amp; Diunggah ke Menu Layanan Informasi / Google Drive)</t>
         </is>
       </c>
     </row>

</xml_diff>